<commit_message>
fidelity: figure retitled 'HGS-M5 vs. M4G (Small Scale)'; M5-λ comparison dropped from bundle (not in thesis)
</commit_message>
<xml_diff>
--- a/experiments/formal/2026-09-18_small_pure_m5_vs_m4g_fidelity/csv/stats_full.xlsx
+++ b/experiments/formal/2026-09-18_small_pure_m5_vs_m4g_fidelity/csv/stats_full.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aesop\Desktop\EE-RAWSim-O_PP\experiments\formal\2026-09-18_small_pure_m5_vs_m4g_fidelity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F58B0D-7200-413A-85BB-C7781F69D25B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{797A9DEC-81AC-42C0-AC2A-849AD0101778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-12645" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="30">
   <si>
     <t>arm</t>
   </si>
@@ -126,13 +126,7 @@
     <t>p</t>
   </si>
   <si>
-    <t>m5_pure_6b vs m5_lambda_6b</t>
-  </si>
-  <si>
     <t>m5_pure_10b vs m4g_10b</t>
-  </si>
-  <si>
-    <t>m5_pure_10b vs m5_lambda_10b</t>
   </si>
 </sst>
 </file>
@@ -2994,7 +2988,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="5" width="18" customWidth="1"/>
@@ -5548,11 +5542,11 @@
         <v>3</v>
       </c>
       <c r="D142">
-        <f>(AVERAGE(per_seed!$D$22:$D$31)-AVERAGE(per_seed!$D$12:$D$21))/AVERAGE(per_seed!$D$12:$D$21)*100</f>
-        <v>-7.7344958514986378E-2</v>
+        <f>(AVERAGE(per_seed!$D$52:$D$61)-AVERAGE(per_seed!$D$32:$D$41))/AVERAGE(per_seed!$D$32:$D$41)*100</f>
+        <v>-6.9993700567044462E-3</v>
       </c>
       <c r="E142">
-        <v>-7.7344958514986378E-2</v>
+        <v>-6.9993700567044462E-3</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -5566,11 +5560,11 @@
         <v>3</v>
       </c>
       <c r="D143">
-        <f>_xlfn.T.TEST(per_seed!$D$12:$D$21,per_seed!$D$22:$D$31,2,1)</f>
-        <v>0.63413155002930433</v>
+        <f>_xlfn.T.TEST(per_seed!$D$32:$D$41,per_seed!$D$52:$D$61,2,1)</f>
+        <v>0.90433842850835133</v>
       </c>
       <c r="E143">
-        <v>0.63413155002934629</v>
+        <v>0.90433842850847856</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -5584,11 +5578,11 @@
         <v>4</v>
       </c>
       <c r="D144">
-        <f>(AVERAGE(per_seed!$E$22:$E$31)-AVERAGE(per_seed!$E$12:$E$21))/AVERAGE(per_seed!$E$12:$E$21)*100</f>
-        <v>-3.2216494845368149E-2</v>
+        <f>(AVERAGE(per_seed!$E$52:$E$61)-AVERAGE(per_seed!$E$32:$E$41))/AVERAGE(per_seed!$E$32:$E$41)*100</f>
+        <v>-1.5017853392144578</v>
       </c>
       <c r="E144">
-        <v>-3.2216494845368149E-2</v>
+        <v>-1.501785339214458</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -5602,11 +5596,11 @@
         <v>4</v>
       </c>
       <c r="D145">
-        <f>_xlfn.T.TEST(per_seed!$E$12:$E$21,per_seed!$E$22:$E$31,2,1)</f>
-        <v>0.85595125270061856</v>
+        <f>_xlfn.T.TEST(per_seed!$E$32:$E$41,per_seed!$E$52:$E$61,2,1)</f>
+        <v>1.1787578138252746E-3</v>
       </c>
       <c r="E145">
-        <v>0.85595125270065231</v>
+        <v>1.1787578138253161E-3</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -5620,11 +5614,11 @@
         <v>5</v>
       </c>
       <c r="D146">
-        <f>(AVERAGE(per_seed!$F$22:$F$31)-AVERAGE(per_seed!$F$12:$F$21))/AVERAGE(per_seed!$F$12:$F$21)*100</f>
-        <v>1.5410958904109588</v>
+        <f>(AVERAGE(per_seed!$F$52:$F$61)-AVERAGE(per_seed!$F$32:$F$41))/AVERAGE(per_seed!$F$32:$F$41)*100</f>
+        <v>-1.5907207953604015</v>
       </c>
       <c r="E146">
-        <v>1.5410958904109591</v>
+        <v>-1.590720795360401</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -5638,11 +5632,11 @@
         <v>5</v>
       </c>
       <c r="D147">
-        <f>_xlfn.T.TEST(per_seed!$F$12:$F$21,per_seed!$F$22:$F$31,2,1)</f>
-        <v>8.8910400668309776E-3</v>
+        <f>_xlfn.T.TEST(per_seed!$F$32:$F$41,per_seed!$F$52:$F$61,2,1)</f>
+        <v>1.4129254523320251E-2</v>
       </c>
       <c r="E147">
-        <v>8.8910400668309793E-3</v>
+        <v>1.412925452332041E-2</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -5656,11 +5650,11 @@
         <v>6</v>
       </c>
       <c r="D148">
-        <f>(AVERAGE(per_seed!$G$22:$G$31)-AVERAGE(per_seed!$G$12:$G$21))/AVERAGE(per_seed!$G$12:$G$21)*100</f>
-        <v>12.288025537404138</v>
+        <f>(AVERAGE(per_seed!$G$52:$G$61)-AVERAGE(per_seed!$G$32:$G$41))/AVERAGE(per_seed!$G$32:$G$41)*100</f>
+        <v>11.018273935911232</v>
       </c>
       <c r="E148">
-        <v>12.28802553740414</v>
+        <v>11.018273935911269</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -5674,11 +5668,11 @@
         <v>6</v>
       </c>
       <c r="D149">
-        <f>_xlfn.T.TEST(per_seed!$G$12:$G$21,per_seed!$G$22:$G$31,2,1)</f>
-        <v>8.1474826483676878E-7</v>
+        <f>_xlfn.T.TEST(per_seed!$G$32:$G$41,per_seed!$G$52:$G$61,2,1)</f>
+        <v>7.5819886318976554E-6</v>
       </c>
       <c r="E149">
-        <v>8.1474826483676073E-7</v>
+        <v>7.5819886318975521E-6</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -5692,11 +5686,11 @@
         <v>7</v>
       </c>
       <c r="D150">
-        <f>(AVERAGE(per_seed!$H$22:$H$31)-AVERAGE(per_seed!$H$12:$H$21))/AVERAGE(per_seed!$H$12:$H$21)*100</f>
-        <v>-9.579230080572966</v>
+        <f>(AVERAGE(per_seed!$H$52:$H$61)-AVERAGE(per_seed!$H$32:$H$41))/AVERAGE(per_seed!$H$32:$H$41)*100</f>
+        <v>-11.355932203389834</v>
       </c>
       <c r="E150">
-        <v>-9.579230080572966</v>
+        <v>-11.35593220338983</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -5710,11 +5704,11 @@
         <v>7</v>
       </c>
       <c r="D151">
-        <f>_xlfn.T.TEST(per_seed!$H$12:$H$21,per_seed!$H$22:$H$31,2,1)</f>
-        <v>1.1931662286760438E-5</v>
+        <f>_xlfn.T.TEST(per_seed!$H$32:$H$41,per_seed!$H$52:$H$61,2,1)</f>
+        <v>3.6740557415890806E-7</v>
       </c>
       <c r="E151">
-        <v>1.193166228676043E-5</v>
+        <v>3.674055741589098E-7</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -5728,11 +5722,11 @@
         <v>8</v>
       </c>
       <c r="D152">
-        <f>(AVERAGE(per_seed!$I$22:$I$31)-AVERAGE(per_seed!$I$12:$I$21))/AVERAGE(per_seed!$I$12:$I$21)*100</f>
-        <v>-10.936365889959946</v>
+        <f>(AVERAGE(per_seed!$I$52:$I$61)-AVERAGE(per_seed!$I$32:$I$41))/AVERAGE(per_seed!$I$32:$I$41)*100</f>
+        <v>-9.9167395917073229</v>
       </c>
       <c r="E152">
-        <v>-10.93636588995993</v>
+        <v>-9.9167395917073229</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -5746,11 +5740,11 @@
         <v>8</v>
       </c>
       <c r="D153">
-        <f>_xlfn.T.TEST(per_seed!$I$12:$I$21,per_seed!$I$22:$I$31,2,1)</f>
-        <v>7.5158002408056447E-7</v>
+        <f>_xlfn.T.TEST(per_seed!$I$32:$I$41,per_seed!$I$52:$I$61,2,1)</f>
+        <v>8.2592912313688074E-6</v>
       </c>
       <c r="E153">
-        <v>7.5158002408053821E-7</v>
+        <v>8.2592912313691868E-6</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -5764,11 +5758,11 @@
         <v>9</v>
       </c>
       <c r="D154">
-        <f>(AVERAGE(per_seed!$J$22:$J$31)-AVERAGE(per_seed!$J$12:$J$21))/AVERAGE(per_seed!$J$12:$J$21)*100</f>
-        <v>-3.181849800478647E-2</v>
+        <f>(AVERAGE(per_seed!$J$52:$J$61)-AVERAGE(per_seed!$J$32:$J$41))/AVERAGE(per_seed!$J$32:$J$41)*100</f>
+        <v>-0.89719675500850304</v>
       </c>
       <c r="E154">
-        <v>-3.181849800478647E-2</v>
+        <v>-0.89719675500852003</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -5782,11 +5776,11 @@
         <v>9</v>
       </c>
       <c r="D155">
-        <f>_xlfn.T.TEST(per_seed!$J$12:$J$21,per_seed!$J$22:$J$31,2,1)</f>
-        <v>0.97582485570997235</v>
+        <f>_xlfn.T.TEST(per_seed!$J$32:$J$41,per_seed!$J$52:$J$61,2,1)</f>
+        <v>0.30978955240123385</v>
       </c>
       <c r="E155">
-        <v>0.97582485570997224</v>
+        <v>0.30978955240123529</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -5800,11 +5794,11 @@
         <v>10</v>
       </c>
       <c r="D156">
-        <f>(AVERAGE(per_seed!$K$22:$K$31)-AVERAGE(per_seed!$K$12:$K$21))/AVERAGE(per_seed!$K$12:$K$21)*100</f>
-        <v>-3.1883594380153659</v>
+        <f>(AVERAGE(per_seed!$K$52:$K$61)-AVERAGE(per_seed!$K$32:$K$41))/AVERAGE(per_seed!$K$32:$K$41)*100</f>
+        <v>-2.7566540051129587</v>
       </c>
       <c r="E156">
-        <v>-3.1883594380153659</v>
+        <v>-2.7566540051129591</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -5818,11 +5812,11 @@
         <v>10</v>
       </c>
       <c r="D157">
-        <f>_xlfn.T.TEST(per_seed!$K$12:$K$21,per_seed!$K$22:$K$31,2,1)</f>
-        <v>1.5732204196688776E-2</v>
+        <f>_xlfn.T.TEST(per_seed!$K$32:$K$41,per_seed!$K$52:$K$61,2,1)</f>
+        <v>3.5171058073491142E-2</v>
       </c>
       <c r="E157">
-        <v>1.5732204196688412E-2</v>
+        <v>3.517105807349144E-2</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -5836,11 +5830,11 @@
         <v>11</v>
       </c>
       <c r="D158">
-        <f>(AVERAGE(per_seed!$L$22:$L$31)-AVERAGE(per_seed!$L$12:$L$21))/AVERAGE(per_seed!$L$12:$L$21)*100</f>
-        <v>-2.8551346372239603</v>
+        <f>(AVERAGE(per_seed!$L$52:$L$61)-AVERAGE(per_seed!$L$32:$L$41))/AVERAGE(per_seed!$L$32:$L$41)*100</f>
+        <v>14.52073342717741</v>
       </c>
       <c r="E158">
-        <v>-2.8551346372239599</v>
+        <v>14.52073342717741</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -5854,11 +5848,11 @@
         <v>11</v>
       </c>
       <c r="D159">
-        <f>_xlfn.T.TEST(per_seed!$L$12:$L$21,per_seed!$L$22:$L$31,2,1)</f>
-        <v>0.24646933520072684</v>
+        <f>_xlfn.T.TEST(per_seed!$L$32:$L$41,per_seed!$L$52:$L$61,2,1)</f>
+        <v>6.6126517436111941E-3</v>
       </c>
       <c r="E159">
-        <v>0.24646933520072689</v>
+        <v>6.6126517436112132E-3</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -5872,11 +5866,11 @@
         <v>12</v>
       </c>
       <c r="D160">
-        <f>(AVERAGE(per_seed!$M$22:$M$31)-AVERAGE(per_seed!$M$12:$M$21))/AVERAGE(per_seed!$M$12:$M$21)*100</f>
-        <v>7.3116234844550032</v>
+        <f>(AVERAGE(per_seed!$M$52:$M$61)-AVERAGE(per_seed!$M$32:$M$41))/AVERAGE(per_seed!$M$32:$M$41)*100</f>
+        <v>1.273173194618973</v>
       </c>
       <c r="E160">
-        <v>7.3116234844550556</v>
+        <v>1.273173194618973</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -5890,731 +5884,11 @@
         <v>12</v>
       </c>
       <c r="D161">
-        <f>_xlfn.T.TEST(per_seed!$M$12:$M$21,per_seed!$M$22:$M$31,2,1)</f>
-        <v>0.54316455242123762</v>
-      </c>
-      <c r="E161">
-        <v>0.54316455242123474</v>
-      </c>
-    </row>
-    <row r="162" spans="1:5">
-      <c r="A162" t="s">
-        <v>26</v>
-      </c>
-      <c r="B162" t="s">
-        <v>30</v>
-      </c>
-      <c r="C162" t="s">
-        <v>3</v>
-      </c>
-      <c r="D162">
-        <f>(AVERAGE(per_seed!$D$52:$D$61)-AVERAGE(per_seed!$D$32:$D$41))/AVERAGE(per_seed!$D$32:$D$41)*100</f>
-        <v>-6.9993700567044462E-3</v>
-      </c>
-      <c r="E162">
-        <v>-6.9993700567044462E-3</v>
-      </c>
-    </row>
-    <row r="163" spans="1:5">
-      <c r="A163" t="s">
-        <v>28</v>
-      </c>
-      <c r="B163" t="s">
-        <v>30</v>
-      </c>
-      <c r="C163" t="s">
-        <v>3</v>
-      </c>
-      <c r="D163">
-        <f>_xlfn.T.TEST(per_seed!$D$32:$D$41,per_seed!$D$52:$D$61,2,1)</f>
-        <v>0.90433842850835133</v>
-      </c>
-      <c r="E163">
-        <v>0.90433842850847856</v>
-      </c>
-    </row>
-    <row r="164" spans="1:5">
-      <c r="A164" t="s">
-        <v>26</v>
-      </c>
-      <c r="B164" t="s">
-        <v>30</v>
-      </c>
-      <c r="C164" t="s">
-        <v>4</v>
-      </c>
-      <c r="D164">
-        <f>(AVERAGE(per_seed!$E$52:$E$61)-AVERAGE(per_seed!$E$32:$E$41))/AVERAGE(per_seed!$E$32:$E$41)*100</f>
-        <v>-1.5017853392144578</v>
-      </c>
-      <c r="E164">
-        <v>-1.501785339214458</v>
-      </c>
-    </row>
-    <row r="165" spans="1:5">
-      <c r="A165" t="s">
-        <v>28</v>
-      </c>
-      <c r="B165" t="s">
-        <v>30</v>
-      </c>
-      <c r="C165" t="s">
-        <v>4</v>
-      </c>
-      <c r="D165">
-        <f>_xlfn.T.TEST(per_seed!$E$32:$E$41,per_seed!$E$52:$E$61,2,1)</f>
-        <v>1.1787578138252746E-3</v>
-      </c>
-      <c r="E165">
-        <v>1.1787578138253161E-3</v>
-      </c>
-    </row>
-    <row r="166" spans="1:5">
-      <c r="A166" t="s">
-        <v>26</v>
-      </c>
-      <c r="B166" t="s">
-        <v>30</v>
-      </c>
-      <c r="C166" t="s">
-        <v>5</v>
-      </c>
-      <c r="D166">
-        <f>(AVERAGE(per_seed!$F$52:$F$61)-AVERAGE(per_seed!$F$32:$F$41))/AVERAGE(per_seed!$F$32:$F$41)*100</f>
-        <v>-1.5907207953604015</v>
-      </c>
-      <c r="E166">
-        <v>-1.590720795360401</v>
-      </c>
-    </row>
-    <row r="167" spans="1:5">
-      <c r="A167" t="s">
-        <v>28</v>
-      </c>
-      <c r="B167" t="s">
-        <v>30</v>
-      </c>
-      <c r="C167" t="s">
-        <v>5</v>
-      </c>
-      <c r="D167">
-        <f>_xlfn.T.TEST(per_seed!$F$32:$F$41,per_seed!$F$52:$F$61,2,1)</f>
-        <v>1.4129254523320251E-2</v>
-      </c>
-      <c r="E167">
-        <v>1.412925452332041E-2</v>
-      </c>
-    </row>
-    <row r="168" spans="1:5">
-      <c r="A168" t="s">
-        <v>26</v>
-      </c>
-      <c r="B168" t="s">
-        <v>30</v>
-      </c>
-      <c r="C168" t="s">
-        <v>6</v>
-      </c>
-      <c r="D168">
-        <f>(AVERAGE(per_seed!$G$52:$G$61)-AVERAGE(per_seed!$G$32:$G$41))/AVERAGE(per_seed!$G$32:$G$41)*100</f>
-        <v>11.018273935911232</v>
-      </c>
-      <c r="E168">
-        <v>11.018273935911269</v>
-      </c>
-    </row>
-    <row r="169" spans="1:5">
-      <c r="A169" t="s">
-        <v>28</v>
-      </c>
-      <c r="B169" t="s">
-        <v>30</v>
-      </c>
-      <c r="C169" t="s">
-        <v>6</v>
-      </c>
-      <c r="D169">
-        <f>_xlfn.T.TEST(per_seed!$G$32:$G$41,per_seed!$G$52:$G$61,2,1)</f>
-        <v>7.5819886318976554E-6</v>
-      </c>
-      <c r="E169">
-        <v>7.5819886318975521E-6</v>
-      </c>
-    </row>
-    <row r="170" spans="1:5">
-      <c r="A170" t="s">
-        <v>26</v>
-      </c>
-      <c r="B170" t="s">
-        <v>30</v>
-      </c>
-      <c r="C170" t="s">
-        <v>7</v>
-      </c>
-      <c r="D170">
-        <f>(AVERAGE(per_seed!$H$52:$H$61)-AVERAGE(per_seed!$H$32:$H$41))/AVERAGE(per_seed!$H$32:$H$41)*100</f>
-        <v>-11.355932203389834</v>
-      </c>
-      <c r="E170">
-        <v>-11.35593220338983</v>
-      </c>
-    </row>
-    <row r="171" spans="1:5">
-      <c r="A171" t="s">
-        <v>28</v>
-      </c>
-      <c r="B171" t="s">
-        <v>30</v>
-      </c>
-      <c r="C171" t="s">
-        <v>7</v>
-      </c>
-      <c r="D171">
-        <f>_xlfn.T.TEST(per_seed!$H$32:$H$41,per_seed!$H$52:$H$61,2,1)</f>
-        <v>3.6740557415890806E-7</v>
-      </c>
-      <c r="E171">
-        <v>3.674055741589098E-7</v>
-      </c>
-    </row>
-    <row r="172" spans="1:5">
-      <c r="A172" t="s">
-        <v>26</v>
-      </c>
-      <c r="B172" t="s">
-        <v>30</v>
-      </c>
-      <c r="C172" t="s">
-        <v>8</v>
-      </c>
-      <c r="D172">
-        <f>(AVERAGE(per_seed!$I$52:$I$61)-AVERAGE(per_seed!$I$32:$I$41))/AVERAGE(per_seed!$I$32:$I$41)*100</f>
-        <v>-9.9167395917073229</v>
-      </c>
-      <c r="E172">
-        <v>-9.9167395917073229</v>
-      </c>
-    </row>
-    <row r="173" spans="1:5">
-      <c r="A173" t="s">
-        <v>28</v>
-      </c>
-      <c r="B173" t="s">
-        <v>30</v>
-      </c>
-      <c r="C173" t="s">
-        <v>8</v>
-      </c>
-      <c r="D173">
-        <f>_xlfn.T.TEST(per_seed!$I$32:$I$41,per_seed!$I$52:$I$61,2,1)</f>
-        <v>8.2592912313688074E-6</v>
-      </c>
-      <c r="E173">
-        <v>8.2592912313691868E-6</v>
-      </c>
-    </row>
-    <row r="174" spans="1:5">
-      <c r="A174" t="s">
-        <v>26</v>
-      </c>
-      <c r="B174" t="s">
-        <v>30</v>
-      </c>
-      <c r="C174" t="s">
-        <v>9</v>
-      </c>
-      <c r="D174">
-        <f>(AVERAGE(per_seed!$J$52:$J$61)-AVERAGE(per_seed!$J$32:$J$41))/AVERAGE(per_seed!$J$32:$J$41)*100</f>
-        <v>-0.89719675500850304</v>
-      </c>
-      <c r="E174">
-        <v>-0.89719675500852003</v>
-      </c>
-    </row>
-    <row r="175" spans="1:5">
-      <c r="A175" t="s">
-        <v>28</v>
-      </c>
-      <c r="B175" t="s">
-        <v>30</v>
-      </c>
-      <c r="C175" t="s">
-        <v>9</v>
-      </c>
-      <c r="D175">
-        <f>_xlfn.T.TEST(per_seed!$J$32:$J$41,per_seed!$J$52:$J$61,2,1)</f>
-        <v>0.30978955240123385</v>
-      </c>
-      <c r="E175">
-        <v>0.30978955240123529</v>
-      </c>
-    </row>
-    <row r="176" spans="1:5">
-      <c r="A176" t="s">
-        <v>26</v>
-      </c>
-      <c r="B176" t="s">
-        <v>30</v>
-      </c>
-      <c r="C176" t="s">
-        <v>10</v>
-      </c>
-      <c r="D176">
-        <f>(AVERAGE(per_seed!$K$52:$K$61)-AVERAGE(per_seed!$K$32:$K$41))/AVERAGE(per_seed!$K$32:$K$41)*100</f>
-        <v>-2.7566540051129587</v>
-      </c>
-      <c r="E176">
-        <v>-2.7566540051129591</v>
-      </c>
-    </row>
-    <row r="177" spans="1:5">
-      <c r="A177" t="s">
-        <v>28</v>
-      </c>
-      <c r="B177" t="s">
-        <v>30</v>
-      </c>
-      <c r="C177" t="s">
-        <v>10</v>
-      </c>
-      <c r="D177">
-        <f>_xlfn.T.TEST(per_seed!$K$32:$K$41,per_seed!$K$52:$K$61,2,1)</f>
-        <v>3.5171058073491142E-2</v>
-      </c>
-      <c r="E177">
-        <v>3.517105807349144E-2</v>
-      </c>
-    </row>
-    <row r="178" spans="1:5">
-      <c r="A178" t="s">
-        <v>26</v>
-      </c>
-      <c r="B178" t="s">
-        <v>30</v>
-      </c>
-      <c r="C178" t="s">
-        <v>11</v>
-      </c>
-      <c r="D178">
-        <f>(AVERAGE(per_seed!$L$52:$L$61)-AVERAGE(per_seed!$L$32:$L$41))/AVERAGE(per_seed!$L$32:$L$41)*100</f>
-        <v>14.52073342717741</v>
-      </c>
-      <c r="E178">
-        <v>14.52073342717741</v>
-      </c>
-    </row>
-    <row r="179" spans="1:5">
-      <c r="A179" t="s">
-        <v>28</v>
-      </c>
-      <c r="B179" t="s">
-        <v>30</v>
-      </c>
-      <c r="C179" t="s">
-        <v>11</v>
-      </c>
-      <c r="D179">
-        <f>_xlfn.T.TEST(per_seed!$L$32:$L$41,per_seed!$L$52:$L$61,2,1)</f>
-        <v>6.6126517436111941E-3</v>
-      </c>
-      <c r="E179">
-        <v>6.6126517436112132E-3</v>
-      </c>
-    </row>
-    <row r="180" spans="1:5">
-      <c r="A180" t="s">
-        <v>26</v>
-      </c>
-      <c r="B180" t="s">
-        <v>30</v>
-      </c>
-      <c r="C180" t="s">
-        <v>12</v>
-      </c>
-      <c r="D180">
-        <f>(AVERAGE(per_seed!$M$52:$M$61)-AVERAGE(per_seed!$M$32:$M$41))/AVERAGE(per_seed!$M$32:$M$41)*100</f>
-        <v>1.273173194618973</v>
-      </c>
-      <c r="E180">
-        <v>1.273173194618973</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5">
-      <c r="A181" t="s">
-        <v>28</v>
-      </c>
-      <c r="B181" t="s">
-        <v>30</v>
-      </c>
-      <c r="C181" t="s">
-        <v>12</v>
-      </c>
-      <c r="D181">
         <f>_xlfn.T.TEST(per_seed!$M$32:$M$41,per_seed!$M$52:$M$61,2,1)</f>
         <v>0.83072781201327817</v>
       </c>
-      <c r="E181">
+      <c r="E161">
         <v>0.8307278120132795</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5">
-      <c r="A182" t="s">
-        <v>26</v>
-      </c>
-      <c r="B182" t="s">
-        <v>31</v>
-      </c>
-      <c r="C182" t="s">
-        <v>3</v>
-      </c>
-      <c r="D182">
-        <f>(AVERAGE(per_seed!$D$52:$D$61)-AVERAGE(per_seed!$D$42:$D$51))/AVERAGE(per_seed!$D$42:$D$51)*100</f>
-        <v>-0.1188561840173422</v>
-      </c>
-      <c r="E182">
-        <v>-0.1188561840173422</v>
-      </c>
-    </row>
-    <row r="183" spans="1:5">
-      <c r="A183" t="s">
-        <v>28</v>
-      </c>
-      <c r="B183" t="s">
-        <v>31</v>
-      </c>
-      <c r="C183" t="s">
-        <v>3</v>
-      </c>
-      <c r="D183">
-        <f>_xlfn.T.TEST(per_seed!$D$42:$D$51,per_seed!$D$52:$D$61,2,1)</f>
-        <v>1.0765027603852948E-4</v>
-      </c>
-      <c r="E183">
-        <v>1.076502760385513E-4</v>
-      </c>
-    </row>
-    <row r="184" spans="1:5">
-      <c r="A184" t="s">
-        <v>26</v>
-      </c>
-      <c r="B184" t="s">
-        <v>31</v>
-      </c>
-      <c r="C184" t="s">
-        <v>4</v>
-      </c>
-      <c r="D184">
-        <f>(AVERAGE(per_seed!$E$52:$E$61)-AVERAGE(per_seed!$E$42:$E$51))/AVERAGE(per_seed!$E$42:$E$51)*100</f>
-        <v>0.39606080068507082</v>
-      </c>
-      <c r="E184">
-        <v>0.39606080068507082</v>
-      </c>
-    </row>
-    <row r="185" spans="1:5">
-      <c r="A185" t="s">
-        <v>28</v>
-      </c>
-      <c r="B185" t="s">
-        <v>31</v>
-      </c>
-      <c r="C185" t="s">
-        <v>4</v>
-      </c>
-      <c r="D185">
-        <f>_xlfn.T.TEST(per_seed!$E$42:$E$51,per_seed!$E$52:$E$61,2,1)</f>
-        <v>2.8683339574939706E-2</v>
-      </c>
-      <c r="E185">
-        <v>2.868333957493762E-2</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5">
-      <c r="A186" t="s">
-        <v>26</v>
-      </c>
-      <c r="B186" t="s">
-        <v>31</v>
-      </c>
-      <c r="C186" t="s">
-        <v>5</v>
-      </c>
-      <c r="D186">
-        <f>(AVERAGE(per_seed!$F$52:$F$61)-AVERAGE(per_seed!$F$42:$F$51))/AVERAGE(per_seed!$F$42:$F$51)*100</f>
-        <v>0.98622683217139162</v>
-      </c>
-      <c r="E186">
-        <v>0.98622683217139162</v>
-      </c>
-    </row>
-    <row r="187" spans="1:5">
-      <c r="A187" t="s">
-        <v>28</v>
-      </c>
-      <c r="B187" t="s">
-        <v>31</v>
-      </c>
-      <c r="C187" t="s">
-        <v>5</v>
-      </c>
-      <c r="D187">
-        <f>_xlfn.T.TEST(per_seed!$F$42:$F$51,per_seed!$F$52:$F$61,2,1)</f>
-        <v>2.38975974278556E-3</v>
-      </c>
-      <c r="E187">
-        <v>2.3897597427854321E-3</v>
-      </c>
-    </row>
-    <row r="188" spans="1:5">
-      <c r="A188" t="s">
-        <v>26</v>
-      </c>
-      <c r="B188" t="s">
-        <v>31</v>
-      </c>
-      <c r="C188" t="s">
-        <v>6</v>
-      </c>
-      <c r="D188">
-        <f>(AVERAGE(per_seed!$G$52:$G$61)-AVERAGE(per_seed!$G$42:$G$51))/AVERAGE(per_seed!$G$42:$G$51)*100</f>
-        <v>11.82487950891527</v>
-      </c>
-      <c r="E188">
-        <v>11.82487950891529</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5">
-      <c r="A189" t="s">
-        <v>28</v>
-      </c>
-      <c r="B189" t="s">
-        <v>31</v>
-      </c>
-      <c r="C189" t="s">
-        <v>6</v>
-      </c>
-      <c r="D189">
-        <f>_xlfn.T.TEST(per_seed!$G$42:$G$51,per_seed!$G$52:$G$61,2,1)</f>
-        <v>3.8752418940396703E-7</v>
-      </c>
-      <c r="E189">
-        <v>3.8752418940396809E-7</v>
-      </c>
-    </row>
-    <row r="190" spans="1:5">
-      <c r="A190" t="s">
-        <v>26</v>
-      </c>
-      <c r="B190" t="s">
-        <v>31</v>
-      </c>
-      <c r="C190" t="s">
-        <v>7</v>
-      </c>
-      <c r="D190">
-        <f>(AVERAGE(per_seed!$H$52:$H$61)-AVERAGE(per_seed!$H$42:$H$51))/AVERAGE(per_seed!$H$42:$H$51)*100</f>
-        <v>-9.6718480138169287</v>
-      </c>
-      <c r="E190">
-        <v>-9.6718480138169287</v>
-      </c>
-    </row>
-    <row r="191" spans="1:5">
-      <c r="A191" t="s">
-        <v>28</v>
-      </c>
-      <c r="B191" t="s">
-        <v>31</v>
-      </c>
-      <c r="C191" t="s">
-        <v>7</v>
-      </c>
-      <c r="D191">
-        <f>_xlfn.T.TEST(per_seed!$H$42:$H$51,per_seed!$H$52:$H$61,2,1)</f>
-        <v>3.5916006526857521E-7</v>
-      </c>
-      <c r="E191">
-        <v>3.591600652685749E-7</v>
-      </c>
-    </row>
-    <row r="192" spans="1:5">
-      <c r="A192" t="s">
-        <v>26</v>
-      </c>
-      <c r="B192" t="s">
-        <v>31</v>
-      </c>
-      <c r="C192" t="s">
-        <v>8</v>
-      </c>
-      <c r="D192">
-        <f>(AVERAGE(per_seed!$I$52:$I$61)-AVERAGE(per_seed!$I$42:$I$51))/AVERAGE(per_seed!$I$42:$I$51)*100</f>
-        <v>-10.554259533494994</v>
-      </c>
-      <c r="E192">
-        <v>-10.55425953349499</v>
-      </c>
-    </row>
-    <row r="193" spans="1:5">
-      <c r="A193" t="s">
-        <v>28</v>
-      </c>
-      <c r="B193" t="s">
-        <v>31</v>
-      </c>
-      <c r="C193" t="s">
-        <v>8</v>
-      </c>
-      <c r="D193">
-        <f>_xlfn.T.TEST(per_seed!$I$42:$I$51,per_seed!$I$52:$I$61,2,1)</f>
-        <v>3.1774501782914263E-7</v>
-      </c>
-      <c r="E193">
-        <v>3.1774501782914639E-7</v>
-      </c>
-    </row>
-    <row r="194" spans="1:5">
-      <c r="A194" t="s">
-        <v>26</v>
-      </c>
-      <c r="B194" t="s">
-        <v>31</v>
-      </c>
-      <c r="C194" t="s">
-        <v>9</v>
-      </c>
-      <c r="D194">
-        <f>(AVERAGE(per_seed!$J$52:$J$61)-AVERAGE(per_seed!$J$42:$J$51))/AVERAGE(per_seed!$J$42:$J$51)*100</f>
-        <v>0.71682711575507185</v>
-      </c>
-      <c r="E194">
-        <v>0.71682711575507185</v>
-      </c>
-    </row>
-    <row r="195" spans="1:5">
-      <c r="A195" t="s">
-        <v>28</v>
-      </c>
-      <c r="B195" t="s">
-        <v>31</v>
-      </c>
-      <c r="C195" t="s">
-        <v>9</v>
-      </c>
-      <c r="D195">
-        <f>_xlfn.T.TEST(per_seed!$J$42:$J$51,per_seed!$J$52:$J$61,2,1)</f>
-        <v>0.2928459305231903</v>
-      </c>
-      <c r="E195">
-        <v>0.29284593052317881</v>
-      </c>
-    </row>
-    <row r="196" spans="1:5">
-      <c r="A196" t="s">
-        <v>26</v>
-      </c>
-      <c r="B196" t="s">
-        <v>31</v>
-      </c>
-      <c r="C196" t="s">
-        <v>10</v>
-      </c>
-      <c r="D196">
-        <f>(AVERAGE(per_seed!$K$52:$K$61)-AVERAGE(per_seed!$K$42:$K$51))/AVERAGE(per_seed!$K$42:$K$51)*100</f>
-        <v>-2.3763459623009937</v>
-      </c>
-      <c r="E196">
-        <v>-2.3763459623009942</v>
-      </c>
-    </row>
-    <row r="197" spans="1:5">
-      <c r="A197" t="s">
-        <v>28</v>
-      </c>
-      <c r="B197" t="s">
-        <v>31</v>
-      </c>
-      <c r="C197" t="s">
-        <v>10</v>
-      </c>
-      <c r="D197">
-        <f>_xlfn.T.TEST(per_seed!$K$42:$K$51,per_seed!$K$52:$K$61,2,1)</f>
-        <v>7.6146051019341148E-3</v>
-      </c>
-      <c r="E197">
-        <v>7.6146051019342492E-3</v>
-      </c>
-    </row>
-    <row r="198" spans="1:5">
-      <c r="A198" t="s">
-        <v>26</v>
-      </c>
-      <c r="B198" t="s">
-        <v>31</v>
-      </c>
-      <c r="C198" t="s">
-        <v>11</v>
-      </c>
-      <c r="D198">
-        <f>(AVERAGE(per_seed!$L$52:$L$61)-AVERAGE(per_seed!$L$42:$L$51))/AVERAGE(per_seed!$L$42:$L$51)*100</f>
-        <v>-5.5487569388230771</v>
-      </c>
-      <c r="E198">
-        <v>-5.5487569388230771</v>
-      </c>
-    </row>
-    <row r="199" spans="1:5">
-      <c r="A199" t="s">
-        <v>28</v>
-      </c>
-      <c r="B199" t="s">
-        <v>31</v>
-      </c>
-      <c r="C199" t="s">
-        <v>11</v>
-      </c>
-      <c r="D199">
-        <f>_xlfn.T.TEST(per_seed!$L$42:$L$51,per_seed!$L$52:$L$61,2,1)</f>
-        <v>0.11417486831017634</v>
-      </c>
-      <c r="E199">
-        <v>0.1141748683101763</v>
-      </c>
-    </row>
-    <row r="200" spans="1:5">
-      <c r="A200" t="s">
-        <v>26</v>
-      </c>
-      <c r="B200" t="s">
-        <v>31</v>
-      </c>
-      <c r="C200" t="s">
-        <v>12</v>
-      </c>
-      <c r="D200">
-        <f>(AVERAGE(per_seed!$M$52:$M$61)-AVERAGE(per_seed!$M$42:$M$51))/AVERAGE(per_seed!$M$42:$M$51)*100</f>
-        <v>17.860141030687156</v>
-      </c>
-      <c r="E200">
-        <v>17.86014103068716</v>
-      </c>
-    </row>
-    <row r="201" spans="1:5">
-      <c r="A201" t="s">
-        <v>28</v>
-      </c>
-      <c r="B201" t="s">
-        <v>31</v>
-      </c>
-      <c r="C201" t="s">
-        <v>12</v>
-      </c>
-      <c r="D201">
-        <f>_xlfn.T.TEST(per_seed!$M$42:$M$51,per_seed!$M$52:$M$61,2,1)</f>
-        <v>4.1237713845622596E-7</v>
-      </c>
-      <c r="E201">
-        <v>4.1237713845622638E-7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>